<commit_message>
vixlens-catalogo 0.9.1: promovix com cores Kodak/Essilor e selo -50% chamativo
Ajustes pedidos em 01/10 sobre a Promovix Outubro:
- Lente pronta Kodak no amarelo Kodak, com a linha Transitions destacada
  (legenda "Transitions · Fotossensível").
- Lente pronta Essilor no cinza-azulado #414B55 da tabela oficial Essilor.
- Selo "REFLECTA −50%" maior: rótulo branco, valor grande em amarelo,
  contorno amarelo, inclinado e com sombra.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plugins/vixlens-catalogo/skills/promovix/modelo/Promovix_modelo.xlsx
+++ b/plugins/vixlens-catalogo/skills/promovix/modelo/Promovix_modelo.xlsx
@@ -458,7 +458,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -1971,7 +1970,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>#006BB2</t>
+          <t>#F7B200</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1999,7 +1998,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>S</t>
         </is>
       </c>
     </row>
@@ -2016,7 +2015,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>#006BB2</t>
+          <t>#414B55</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -2048,6 +2047,7 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
@@ -6723,6 +6723,11 @@
       <c r="P116" s="6" t="n">
         <v>175</v>
       </c>
+      <c r="U116" t="inlineStr">
+        <is>
+          <t>FOTO</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">

</xml_diff>

<commit_message>
vixlens-catalogo 0.10.0: promovix com pílula Transitions, selo de montagem e Solar compacta
Ajustes da Promovix Outubro pedidos pelo Otávio em 01/10/2026:
- "Transitions ..." no nome do produto vira pílula (Gen S em degradê,
  XTRActive cinza-escuro com texto branco); a linha 8365 deixa o destaque FOTO
- selo "MONTAGEM LENTE PRONTA R$15" no cabeçalho da família (selo_montagem),
  no lugar da faixa preta de montagem
- bloco compacto em 2 colunas para família curta (compacta), usado na Solar,
  que passou para a página da lente pronta
- +10 px de padding no topo das tabelas com o adesivo REFLECTA -50%
- respiro das linhas até 6 px; Excel modelo com a nova distribuição de páginas

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plugins/vixlens-catalogo/skills/promovix/modelo/Promovix_modelo.xlsx
+++ b/plugins/vixlens-catalogo/skills/promovix/modelo/Promovix_modelo.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -525,6 +525,20 @@
       <c r="A12" t="inlineStr">
         <is>
           <t>Preço é decisão de quem preenche. A skill lê, confere e monta — não inventa valor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Transitions no nome do produto vira pílula automaticamente: Gen S (e demais) em degradê, XTRActive em cinza-escuro com texto branco. Não precisa marcar nada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>destaque FOTO não é para Transitions: a pílula já identifica. Use FOTO só em fotossensível de outra marca (Optview Sun+, Resina Foto).</t>
         </is>
       </c>
     </row>
@@ -539,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -883,6 +897,24 @@
       <c r="C20" s="4" t="inlineStr">
         <is>
           <t>Adesivo preto sobre as colunas em promoção (colunas_promo). Vazio = sem adesivo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>montagem_selo</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>MONTAGEM
+LENTE PRONTA</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Selo de montagem no cabeçalho (selo_montagem = S): rótulo em branco ao lado do valor de montagem_destaque.</t>
         </is>
       </c>
     </row>
@@ -933,7 +965,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>Blocos especiais: CAPA, FAIXA_50, FAIXA_MONTAGEM, VIXCLUB. O resto é nome de família (aba Familias). A ordem das linhas é a ordem na página.</t>
+          <t>Blocos especiais: CAPA, FAIXA_50, FAIXA_MONTAGEM, VIXCLUB. O resto é nome de família (aba Familias). A ordem das linhas é a ordem na página. A montagem de lente pronta hoje vai como selo no cabeçalho (selo_montagem na aba Familias), não como faixa.</t>
         </is>
       </c>
     </row>
@@ -973,7 +1005,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>SOLAR ACABADA</t>
+          <t>VIXCLUB</t>
         </is>
       </c>
     </row>
@@ -1013,7 +1045,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>KODAK NETWORK UHD</t>
+          <t>FAIXA_50</t>
         </is>
       </c>
     </row>
@@ -1023,7 +1055,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>KODAK SOFTWEAR</t>
+          <t>KODAK NETWORK UHD</t>
         </is>
       </c>
     </row>
@@ -1033,7 +1065,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>VIXCLUB</t>
+          <t>KODAK SOFTWEAR</t>
         </is>
       </c>
     </row>
@@ -1083,7 +1115,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>FAIXA_MONTAGEM</t>
+          <t>OPTVIEW</t>
         </is>
       </c>
     </row>
@@ -1093,17 +1125,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>OPTVIEW</t>
+          <t>MULTIFOCAL ACABADA</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>MULTIFOCAL ACABADA</t>
+          <t>LENTE PRONTA KODAK</t>
         </is>
       </c>
     </row>
@@ -1113,7 +1145,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>FAIXA_MONTAGEM</t>
+          <t>LENTE PRONTA ESSILOR</t>
         </is>
       </c>
     </row>
@@ -1123,20 +1155,11 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>LENTE PRONTA KODAK</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="n">
-        <v>8</v>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>LENTE PRONTA ESSILOR</t>
-        </is>
-      </c>
-    </row>
+          <t>SOLAR ACABADA</t>
+        </is>
+      </c>
+    </row>
+    <row r="22"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1148,7 +1171,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L25"/>
+  <dimension ref="A1:N27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1163,6 +1186,8 @@
     <col width="16" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1226,6 +1251,16 @@
           <t>legenda_destaque</t>
         </is>
       </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>selo_montagem</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>compacta</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1276,6 +1311,16 @@
           <t>N</t>
         </is>
       </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1326,6 +1371,16 @@
           <t>N</t>
         </is>
       </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1376,6 +1431,16 @@
           <t>N</t>
         </is>
       </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1426,6 +1491,16 @@
           <t>N</t>
         </is>
       </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1481,6 +1556,16 @@
           <t>N</t>
         </is>
       </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1536,6 +1621,16 @@
           <t>N</t>
         </is>
       </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1591,6 +1686,16 @@
           <t>N</t>
         </is>
       </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1646,6 +1751,16 @@
           <t>N</t>
         </is>
       </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1701,6 +1816,16 @@
           <t>N</t>
         </is>
       </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1756,6 +1881,16 @@
           <t>N</t>
         </is>
       </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1811,6 +1946,16 @@
           <t>N</t>
         </is>
       </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1866,6 +2011,16 @@
           <t>N</t>
         </is>
       </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1911,6 +2066,16 @@
           <t>S</t>
         </is>
       </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1956,6 +2121,16 @@
           <t>S</t>
         </is>
       </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2001,6 +2176,16 @@
           <t>S</t>
         </is>
       </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2042,6 +2227,16 @@
         <v>95</v>
       </c>
       <c r="L17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -2093,7 +2288,21 @@
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>legenda_destaque = S: pílulas "Fotossensível" / "RX" no cabeçalho quando houver linhas destacadas.</t>
+          <t>legenda_destaque = S: pílulas "Fotossensível" / "RX" no cabeçalho quando houver linhas destacadas; família com Transitions ganha a legenda "Transitions · Fotossensível" em degradê.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>selo_montagem = S: selo preto "MONTAGEM LENTE PRONTA R$15" no canto direito do cabeçalho (textos montagem_selo e montagem_destaque do Config).</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>compacta = S: bloco compacto em 2 colunas (código, nome, cor, preço), sem cabeçalho grande — para família curta e de pouco peso, como a Solar. Só 1 coluna de preço.</t>
         </is>
       </c>
     </row>
@@ -6723,11 +6932,6 @@
       <c r="P116" s="6" t="n">
         <v>175</v>
       </c>
-      <c r="U116" t="inlineStr">
-        <is>
-          <t>FOTO</t>
-        </is>
-      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">

</xml_diff>

<commit_message>
promovix: vigência 06/10 a 30/11 no modelo com combo
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plugins/vixlens-catalogo/skills/promovix/modelo/Promovix_modelo.xlsx
+++ b/plugins/vixlens-catalogo/skills/promovix/modelo/Promovix_modelo.xlsx
@@ -920,7 +920,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:C23"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -928,6 +928,7 @@
     <col width="92" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -942,6 +943,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
@@ -1009,6 +1011,7 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="B12" s="3" t="inlineStr">
         <is>
@@ -1064,6 +1067,7 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
     <row r="18">
       <c r="B18" s="3" t="inlineStr">
         <is>
@@ -1724,33 +1728,21 @@
           <t>FAMÍLIA</t>
         </is>
       </c>
-      <c r="B1" s="17" t="n"/>
-      <c r="C1" s="17" t="n"/>
-      <c r="D1" s="17" t="n"/>
       <c r="E1" s="16" t="inlineStr">
         <is>
           <t>COLUNAS DE PREÇO</t>
         </is>
       </c>
-      <c r="F1" s="17" t="n"/>
-      <c r="G1" s="17" t="n"/>
       <c r="H1" s="16" t="inlineStr">
         <is>
           <t>LAYOUT</t>
         </is>
       </c>
-      <c r="I1" s="17" t="n"/>
-      <c r="J1" s="17" t="n"/>
-      <c r="K1" s="17" t="n"/>
-      <c r="L1" s="17" t="n"/>
-      <c r="M1" s="17" t="n"/>
-      <c r="N1" s="17" t="n"/>
       <c r="O1" s="16" t="inlineStr">
         <is>
           <t>CONFERÊNCIA</t>
         </is>
       </c>
-      <c r="P1" s="17" t="n"/>
     </row>
     <row r="2" ht="44" customHeight="1">
       <c r="A2" s="9" t="inlineStr">
@@ -4160,39 +4152,21 @@
           <t>PRODUTO</t>
         </is>
       </c>
-      <c r="B1" s="17" t="n"/>
-      <c r="C1" s="17" t="n"/>
-      <c r="D1" s="17" t="n"/>
       <c r="E1" s="16" t="inlineStr">
         <is>
           <t>MARCAÇÕES</t>
         </is>
       </c>
-      <c r="F1" s="17" t="n"/>
-      <c r="G1" s="17" t="n"/>
-      <c r="H1" s="17" t="n"/>
-      <c r="I1" s="17" t="n"/>
       <c r="J1" s="16" t="inlineStr">
         <is>
           <t>DISPONIBILIDADE</t>
         </is>
       </c>
-      <c r="K1" s="17" t="n"/>
-      <c r="L1" s="17" t="n"/>
-      <c r="M1" s="17" t="n"/>
-      <c r="N1" s="17" t="n"/>
-      <c r="O1" s="17" t="n"/>
-      <c r="P1" s="17" t="n"/>
       <c r="Q1" s="16" t="inlineStr">
         <is>
           <t>PREÇOS</t>
         </is>
       </c>
-      <c r="R1" s="17" t="n"/>
-      <c r="S1" s="17" t="n"/>
-      <c r="T1" s="17" t="n"/>
-      <c r="U1" s="17" t="n"/>
-      <c r="V1" s="17" t="n"/>
       <c r="W1" s="16" t="inlineStr">
         <is>
           <t>CORES TRANSITIONS / SOLAR</t>
@@ -20840,7 +20814,6 @@
           <t>ORDEM DAS PÁGINAS</t>
         </is>
       </c>
-      <c r="B1" s="17" t="n"/>
       <c r="C1" s="16" t="inlineStr">
         <is>
           <t>CONFERÊNCIA</t>

</xml_diff>